<commit_message>
Updated project name to college compass
</commit_message>
<xml_diff>
--- a/students/alex-sample/output/Alex - US College Selection.xlsx
+++ b/students/alex-sample/output/Alex - US College Selection.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="College Selection - Business" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="College Selection - Business" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA33"/>
+  <dimension ref="A1:AC39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -464,6 +464,8 @@
       <c r="Y1" t="inlineStr"/>
       <c r="Z1" t="inlineStr"/>
       <c r="AA1" t="inlineStr"/>
+      <c r="AB1" t="inlineStr"/>
+      <c r="AC1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
@@ -493,6 +495,8 @@
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -534,6 +538,8 @@
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -570,7 +576,9 @@
       <c r="X4" s="1" t="inlineStr"/>
       <c r="Y4" s="1" t="inlineStr"/>
       <c r="Z4" s="1" t="inlineStr"/>
-      <c r="AA4" s="1" t="n"/>
+      <c r="AA4" s="1" t="inlineStr"/>
+      <c r="AB4" s="1" t="inlineStr"/>
+      <c r="AC4" s="1" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -611,6 +619,8 @@
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -647,6 +657,8 @@
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -691,6 +703,8 @@
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -727,6 +741,8 @@
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -767,6 +783,8 @@
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -803,6 +821,8 @@
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
@@ -832,6 +852,8 @@
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -865,6 +887,8 @@
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -901,6 +925,8 @@
       <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -937,6 +963,8 @@
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -973,6 +1001,8 @@
       <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
@@ -1002,6 +1032,8 @@
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1036,105 +1068,115 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
+          <t>Data Quality</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Test Optional</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
           <t>Program Admit Type</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Program Requirements</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Student Meets Program Req?</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Program Admit Notes</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>GPA Mid-50% Range</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>GPA vs Mid-50%</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="O17" s="2" t="inlineStr">
         <is>
           <t>SAT Mid-50% Range</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="P17" s="2" t="inlineStr">
         <is>
           <t>SAT vs Mid-50% (effective)</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr">
+      <c r="Q17" s="2" t="inlineStr">
         <is>
           <t>ACT Mid-50% Range</t>
         </is>
       </c>
-      <c r="P17" s="2" t="inlineStr">
+      <c r="R17" s="2" t="inlineStr">
         <is>
           <t>ACT vs Mid-50% (effective)</t>
         </is>
       </c>
-      <c r="Q17" s="2" t="inlineStr">
+      <c r="S17" s="2" t="inlineStr">
         <is>
           <t>Early Action Deadline</t>
         </is>
       </c>
-      <c r="R17" s="2" t="inlineStr">
+      <c r="T17" s="2" t="inlineStr">
         <is>
           <t>Early Decision Deadline</t>
         </is>
       </c>
-      <c r="S17" s="2" t="inlineStr">
+      <c r="U17" s="2" t="inlineStr">
         <is>
           <t>Regular Decision Deadline</t>
         </is>
       </c>
-      <c r="T17" s="2" t="inlineStr">
+      <c r="V17" s="2" t="inlineStr">
         <is>
           <t>ED Binding</t>
         </is>
       </c>
-      <c r="U17" s="2" t="inlineStr">
+      <c r="W17" s="2" t="inlineStr">
         <is>
           <t>Within Budget</t>
         </is>
       </c>
-      <c r="V17" s="2" t="inlineStr">
+      <c r="X17" s="2" t="inlineStr">
         <is>
           <t>Apply Fall 2026</t>
         </is>
       </c>
-      <c r="W17" s="2" t="inlineStr">
+      <c r="Y17" s="2" t="inlineStr">
         <is>
           <t>Accept Rate (University General)</t>
         </is>
       </c>
-      <c r="X17" s="2" t="inlineStr">
+      <c r="Z17" s="2" t="inlineStr">
         <is>
           <t>Accept Rate (Business Program)</t>
         </is>
       </c>
-      <c r="Y17" s="2" t="inlineStr">
+      <c r="AA17" s="2" t="inlineStr">
         <is>
           <t>Business Program Notes</t>
         </is>
       </c>
-      <c r="Z17" s="2" t="inlineStr">
+      <c r="AB17" s="2" t="inlineStr">
         <is>
           <t>Accept Rate Source</t>
         </is>
       </c>
-      <c r="AA17" s="2" t="inlineStr">
+      <c r="AC17" s="2" t="inlineStr">
         <is>
           <t>US News Rankings Source</t>
         </is>
@@ -1173,34 +1215,34 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>No published program mid-50%; general university admission. No EA/ED.</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="M18" t="inlineStr">
         <is>
           <t>—</t>
@@ -1221,49 +1263,59 @@
           <t>—</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
         <is>
           <t>See admissions site</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="V18" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="W18" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
+      <c r="X18" t="inlineStr">
         <is>
           <t>Yes — Safety (top interest)</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr">
+      <c r="Y18" t="inlineStr">
         <is>
           <t>74.4%</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr">
+      <c r="Z18" t="inlineStr">
         <is>
           <t>Not yet researched</t>
         </is>
       </c>
-      <c r="Y18" t="inlineStr">
+      <c r="AA18" t="inlineStr">
         <is>
           <t>In-state tuition $39,800/year — Ohio resident.</t>
         </is>
       </c>
-      <c r="Z18" t="inlineStr">
+      <c r="AB18" t="inlineStr">
         <is>
           <t>Auto stub — run scoped research for program-level rate (General: https://www.onu.edu/ | Business: https://www.onu.edu/)</t>
         </is>
       </c>
-      <c r="AA18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1298,92 +1350,102 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>Mid-50% columns = university-wide (not College of Business). No EA/ED.</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="M19" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
           <t>1230–1318</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="P19" t="inlineStr">
         <is>
           <t>In mid-50%</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>22–27</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="R19" t="inlineStr">
         <is>
           <t>In mid-50%</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr">
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
         <is>
           <t>See admissions site</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="V19" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="W19" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="X19" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W19" t="inlineStr">
+      <c r="Y19" t="inlineStr">
         <is>
           <t>80%</t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr">
+      <c r="AA19" t="inlineStr">
         <is>
           <t>College of Business Administration (CBA) — Wittich Hall. No separate freshman admission. Rolling admissions, Feb 1 priority. MN-WI reciprocity tuition for MN residents.</t>
         </is>
       </c>
-      <c r="Z19" t="inlineStr">
+      <c r="AB19" t="inlineStr">
         <is>
           <t>No separate admission process (General: https://www.uwlax.edu/link/962fb257e7b84e7f884c9599df23a411.aspx)</t>
         </is>
       </c>
-      <c r="AA19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1418,92 +1480,102 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>Mid-50% columns = university-wide (not College of Business). No EA/ED.</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="M20" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
           <t>1100–1320</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>In mid-50%</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>21–26</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="R20" t="inlineStr">
         <is>
           <t>In mid-50%</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr">
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr">
         <is>
           <t>See admissions site</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr">
+      <c r="V20" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="W20" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
+      <c r="X20" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W20" t="inlineStr">
+      <c r="Y20" t="inlineStr">
         <is>
           <t>87.8%</t>
         </is>
       </c>
-      <c r="Y20" t="inlineStr">
+      <c r="AA20" t="inlineStr">
         <is>
           <t>College of Business — AACSB accredited. MN-WI reciprocity tuition for MN residents.</t>
         </is>
       </c>
-      <c r="Z20" t="inlineStr">
+      <c r="AB20" t="inlineStr">
         <is>
           <t>No separate admission process (General: https://www.collegedata.com/college/University-of-Wisconsin-Eau-Claire)</t>
         </is>
       </c>
-      <c r="AA20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1538,34 +1610,34 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>Mid-50% columns = university-wide (not College of Business). No EA/ED.</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="M21" t="inlineStr">
         <is>
           <t>—</t>
@@ -1578,52 +1650,62 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
           <t>20–25</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="R21" t="inlineStr">
         <is>
           <t>Above (+1 vs high)</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr">
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr">
         <is>
           <t>Sep 1</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
+      <c r="V21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="W21" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr">
+      <c r="X21" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W21" t="inlineStr">
+      <c r="Y21" t="inlineStr">
         <is>
           <t>85%</t>
         </is>
       </c>
-      <c r="Y21" t="inlineStr">
+      <c r="AA21" t="inlineStr">
         <is>
           <t>School of Management — 10 bachelor degrees including Business Administration and Supply Chain Management. No confirmed AACSB accreditation. Rolling admissions; Dec 1 merit scholarship priority.</t>
         </is>
       </c>
-      <c r="Z21" t="inlineStr">
+      <c r="AB21" t="inlineStr">
         <is>
           <t>No separate admission process (General: https://www.appily.com/colleges/university-of-wisconsin-stout)</t>
         </is>
       </c>
-      <c r="AA21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1658,92 +1740,102 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>Mid-50% columns = university-wide (not College of Business). No EA/ED.</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="M22" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
           <t>940–1170</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>Above (+80 vs high)</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>18–24</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="R22" t="inlineStr">
         <is>
           <t>Above (+2 vs high)</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr">
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
         <is>
           <t>See admissions site</t>
         </is>
       </c>
-      <c r="T22" t="inlineStr">
+      <c r="V22" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="W22" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr">
+      <c r="X22" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W22" t="inlineStr">
+      <c r="Y22" t="inlineStr">
         <is>
           <t>94%</t>
         </is>
       </c>
-      <c r="Y22" t="inlineStr">
+      <c r="AA22" t="inlineStr">
         <is>
           <t>College of Business and Economics (COBE) — AACSB accredited (top 1%), Wisconsin largest business school, 5,028 students, 15 majors. No separate admission. MN-WI reciprocity tuition for MN residents.</t>
         </is>
       </c>
-      <c r="Z22" t="inlineStr">
+      <c r="AB22" t="inlineStr">
         <is>
           <t>No separate admission process (General: https://www.collegedata.com/college/University-of-Wisconsin-Whitewater)</t>
         </is>
       </c>
-      <c r="AA22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1778,34 +1870,34 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>No published program mid-50%; general university admission. No EA/ED.</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="M23" t="inlineStr">
         <is>
           <t>—</t>
@@ -1826,49 +1918,59 @@
           <t>—</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr">
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr">
         <is>
           <t>See admissions site</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr">
+      <c r="V23" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="W23" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr">
+      <c r="X23" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W23" t="inlineStr">
+      <c r="Y23" t="inlineStr">
         <is>
           <t>89.4%</t>
         </is>
       </c>
-      <c r="X23" t="inlineStr">
+      <c r="Z23" t="inlineStr">
         <is>
           <t>Not yet researched</t>
         </is>
       </c>
-      <c r="Y23" t="inlineStr">
+      <c r="AA23" t="inlineStr">
         <is>
           <t>Out-of-state tuition $17,603/year.</t>
         </is>
       </c>
-      <c r="Z23" t="inlineStr">
+      <c r="AB23" t="inlineStr">
         <is>
           <t>Auto stub — run scoped research for program-level rate (General: https://www.uwplatt.edu/ | Business: https://www.uwplatt.edu/)</t>
         </is>
       </c>
-      <c r="AA23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1903,34 +2005,34 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>No published program mid-50%; general university admission. No EA/ED.</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="M24" t="inlineStr">
         <is>
           <t>—</t>
@@ -1951,49 +2053,59 @@
           <t>—</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr">
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr">
         <is>
           <t>See admissions site</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr">
+      <c r="V24" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="W24" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr">
+      <c r="X24" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W24" t="inlineStr">
+      <c r="Y24" t="inlineStr">
         <is>
           <t>91.8%</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr">
+      <c r="Z24" t="inlineStr">
         <is>
           <t>Not yet researched</t>
         </is>
       </c>
-      <c r="Y24" t="inlineStr">
+      <c r="AA24" t="inlineStr">
         <is>
           <t>Out-of-state tuition $18,508/year.</t>
         </is>
       </c>
-      <c r="Z24" t="inlineStr">
+      <c r="AB24" t="inlineStr">
         <is>
           <t>Auto stub — run scoped research for program-level rate (General: https://www.uwsp.edu/ | Business: https://www.uwsp.edu/)</t>
         </is>
       </c>
-      <c r="AA24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2028,34 +2140,34 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>No published program mid-50%; general university admission. No EA/ED.</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="M25" t="inlineStr">
         <is>
           <t>—</t>
@@ -2076,49 +2188,59 @@
           <t>—</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr">
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr">
         <is>
           <t>See admissions site</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr">
+      <c r="V25" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="W25" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V25" t="inlineStr">
+      <c r="X25" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W25" t="inlineStr">
+      <c r="Y25" t="inlineStr">
         <is>
           <t>81.7%</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr">
+      <c r="Z25" t="inlineStr">
         <is>
           <t>Not yet researched</t>
         </is>
       </c>
-      <c r="Y25" t="inlineStr">
+      <c r="AA25" t="inlineStr">
         <is>
           <t>Out-of-state tuition $17,470/year.</t>
         </is>
       </c>
-      <c r="Z25" t="inlineStr">
+      <c r="AB25" t="inlineStr">
         <is>
           <t>Auto stub — run scoped research for program-level rate (General: https://www.uwrf.edu/ | Business: https://www.uwrf.edu/)</t>
         </is>
       </c>
-      <c r="AA25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2153,34 +2275,34 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>No published program mid-50%; general university admission. No EA/ED.</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="M26" t="inlineStr">
         <is>
           <t>—</t>
@@ -2201,54 +2323,64 @@
           <t>—</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr">
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr">
         <is>
           <t>See admissions site</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr">
+      <c r="V26" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="W26" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr">
+      <c r="X26" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W26" t="inlineStr">
+      <c r="Y26" t="inlineStr">
         <is>
           <t>88.6%</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr">
+      <c r="Z26" t="inlineStr">
         <is>
           <t>Not yet researched</t>
         </is>
       </c>
-      <c r="Y26" t="inlineStr">
+      <c r="AA26" t="inlineStr">
         <is>
           <t>Out-of-state tuition $17,288/year.</t>
         </is>
       </c>
-      <c r="Z26" t="inlineStr">
+      <c r="AB26" t="inlineStr">
         <is>
           <t>Auto stub — run scoped research for program-level rate (General: https://www.uwgb.edu/ | Business: https://www.uwgb.edu/)</t>
         </is>
       </c>
-      <c r="AA26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Iowa State University</t>
+          <t>Youngstown State University</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2258,12 +2390,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>111 (national)</t>
+          <t>R-MW #99 (regional)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>$28,881</t>
+          <t>$11,113</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2278,92 +2410,107 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Mid-50% columns = university-wide (not College of Business). No EA/ED.</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No published program mid-50%; general university admission. No EA/ED.</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>1130–1350</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>In mid-50%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>21–28</t>
+          <t>—</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>In mid-50%</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr">
         <is>
           <t>See admissions site</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr">
+      <c r="V27" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="W27" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr">
+      <c r="X27" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W27" t="inlineStr">
-        <is>
-          <t>89%</t>
-        </is>
-      </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Ivy College of Business — direct admission, indicate business on main app. No separate application. Fully rolling admissions, no closing date.</t>
+          <t>84.5%</t>
         </is>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t>Direct admission — declare business on main app. No separate rate. (General: https://www.ir.iastate.edu/files/documents/cds/CDS-24-25.pdf)</t>
-        </is>
-      </c>
-      <c r="AA27" t="inlineStr"/>
+          <t>Not yet researched</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>In-state tuition $11,113/year — Ohio resident.</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>Auto stub — run scoped research for program-level rate (General: https://ysu.edu/ | Business: https://ysu.edu/)</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2398,34 +2545,34 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>No published program mid-50%; general university admission. No EA/ED.</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="M28" t="inlineStr">
         <is>
           <t>—</t>
@@ -2446,49 +2593,59 @@
           <t>—</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr">
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr">
         <is>
           <t>See admissions site</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr">
+      <c r="V28" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="W28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr">
+      <c r="X28" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W28" t="inlineStr">
+      <c r="Y28" t="inlineStr">
         <is>
           <t>75.4%</t>
         </is>
       </c>
-      <c r="X28" t="inlineStr">
+      <c r="Z28" t="inlineStr">
         <is>
           <t>Not yet researched</t>
         </is>
       </c>
-      <c r="Y28" t="inlineStr">
+      <c r="AA28" t="inlineStr">
         <is>
           <t>Out-of-state tuition $17,429/year.</t>
         </is>
       </c>
-      <c r="Z28" t="inlineStr">
+      <c r="AB28" t="inlineStr">
         <is>
           <t>Auto stub — run scoped research for program-level rate (General: https://www.uwp.edu/ | Business: https://www.uwp.edu/)</t>
         </is>
       </c>
-      <c r="AA28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2523,34 +2680,34 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>No published program mid-50%; general university admission. No EA/ED.</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="M29" t="inlineStr">
         <is>
           <t>—</t>
@@ -2571,74 +2728,84 @@
           <t>—</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr">
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr">
         <is>
           <t>See admissions site</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr">
+      <c r="V29" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="W29" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V29" t="inlineStr">
+      <c r="X29" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W29" t="inlineStr">
+      <c r="Y29" t="inlineStr">
         <is>
           <t>93.0%</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr">
+      <c r="Z29" t="inlineStr">
         <is>
           <t>Not yet researched</t>
         </is>
       </c>
-      <c r="Y29" t="inlineStr">
+      <c r="AA29" t="inlineStr">
         <is>
           <t>Out-of-state tuition $16,726/year.</t>
         </is>
       </c>
-      <c r="Z29" t="inlineStr">
+      <c r="AB29" t="inlineStr">
         <is>
           <t>Auto stub — run scoped research for program-level rate (General: https://www.uwsuper.edu/ | Business: https://www.uwsuper.edu/)</t>
         </is>
       </c>
-      <c r="AA29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>University of Wisconsin-Milwaukee</t>
+          <t>Miami University-Oxford</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>301 (national)</t>
+          <t>143 (national)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>$23,516</t>
+          <t>$18,161</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>$15,014</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2648,34 +2815,34 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>No published program mid-50%; general university admission. No EA/ED.</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="M30" t="inlineStr">
         <is>
           <t>—</t>
@@ -2696,49 +2863,64 @@
           <t>—</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr">
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr">
         <is>
           <t>See admissions site</t>
         </is>
       </c>
-      <c r="T30" t="inlineStr">
+      <c r="V30" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="W30" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V30" t="inlineStr">
+      <c r="X30" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W30" t="inlineStr">
-        <is>
-          <t>97%</t>
-        </is>
-      </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Sheldon B. Lubar College of Business. No separate admission. Rolling admissions. MN-WI reciprocity tuition for MN residents.</t>
+          <t>75.4%</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>No separate admission process (General: https://www.collegedata.com/college/University-of-Wisconsin-Milwaukee)</t>
-        </is>
-      </c>
-      <c r="AA30" t="inlineStr"/>
+          <t>Not yet researched</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>In-state tuition $18,161/year — Ohio resident.</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>Auto stub — run scoped research for program-level rate (General: https://miamioh.edu/ | Business: https://miamioh.edu/)</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>University of Wisconsin-Oshkosh</t>
+          <t>Kent State University at Kent</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2748,17 +2930,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>352 (national)</t>
+          <t>232 (national)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>$16,444</t>
+          <t>$13,232</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>$14,305</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2768,32 +2950,32 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>Mid-50% columns = university-wide (not College of Business). No EA/ED.</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No published program mid-50%; general university admission. No EA/ED.</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2808,57 +2990,72 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>19–24</t>
+          <t>—</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>Above (+2 vs high)</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr">
         <is>
           <t>See admissions site</t>
         </is>
       </c>
-      <c r="T31" t="inlineStr">
+      <c r="V31" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
+      <c r="W31" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V31" t="inlineStr">
+      <c r="X31" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W31" t="inlineStr">
-        <is>
-          <t>87%</t>
-        </is>
-      </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>AACSB-accredited College of Business. 10 undergraduate majors. No separate admission. Rolling admissions.</t>
+          <t>86.3%</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>No separate admission process (General: https://www.appily.com/colleges/university-of-wisconsin-oshkosh)</t>
-        </is>
-      </c>
-      <c r="AA31" t="inlineStr"/>
+          <t>Not yet researched</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>In-state tuition $13,232/year — Ohio resident.</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>Auto stub — run scoped research for program-level rate (General: https://www.kent.edu/ | Business: https://www.kent.edu/)</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>North Dakota State University-Main Campus</t>
+          <t>University of Toledo</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2868,17 +3065,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>373 (national)</t>
+          <t>293 (national)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>$9,868</t>
+          <t>$12,744</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>$25,648</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2888,97 +3085,112 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>Mid-50% columns = university-wide (not College of Business). No EA/ED.</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No published program mid-50%; general university admission. No EA/ED.</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>1010–1280</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>In mid-50%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>19–25</t>
+          <t>—</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>Above (+1 vs high)</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>Aug 1</t>
-        </is>
-      </c>
-      <c r="T32" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>See admissions site</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
+      <c r="W32" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V32" t="inlineStr">
+      <c r="X32" t="inlineStr">
         <is>
           <t>Yes — Safety</t>
         </is>
       </c>
-      <c r="W32" t="inlineStr">
-        <is>
-          <t>95%</t>
-        </is>
-      </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>College of Business — Barry Hall, downtown Fargo. 8 undergraduate majors. No separate admission requirements. ND reciprocity tuition for MN residents.</t>
+          <t>92.0%</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>No separate admission process (General: https://www.appily.com/colleges/north-dakota-state-university-main-campus)</t>
-        </is>
-      </c>
-      <c r="AA32" t="inlineStr"/>
+          <t>Not yet researched</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>In-state tuition $12,744/year — Ohio resident.</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>Auto stub — run scoped research for program-level rate (General: https://www.utoledo.edu/ | Business: https://www.utoledo.edu/)</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Purdue University-Main Campus</t>
+          <t>University of Wisconsin-Milwaukee</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2988,116 +3200,922 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>301 (national)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>$19,984</t>
+          <t>$23,516</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$15,014</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
           <t>University general only</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
         <is>
           <t>University admit only</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>No published program mid-50%; general university admission. No EA/ED.</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>See admissions site</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>Yes — Safety</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>97%</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>Sheldon B. Lubar College of Business. No separate admission. Rolling admissions. MN-WI reciprocity tuition for MN residents.</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>No separate admission process (General: https://www.collegedata.com/college/University-of-Wisconsin-Milwaukee)</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Cleveland State University</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>343 (national)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>$12,988</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>University general only</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>University admit only</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>No published program mid-50%; general university admission. No EA/ED.</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>See admissions site</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>Yes — Safety</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>91.3%</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>Not yet researched</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>In-state tuition $12,988/year — Ohio resident.</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>Auto stub — run scoped research for program-level rate (General: https://www.csuohio.edu/ | Business: https://www.csuohio.edu/)</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>University of Wisconsin-Oshkosh</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>352 (national)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>$16,444</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>$14,305</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>University general only</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>University admit only</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>Mid-50% columns = university-wide (not College of Business). No EA/ED.</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>3.70–4.00</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>Below (-0.25 vs low)</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>1220–1480</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>19–24</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Above (+2 vs high)</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>See admissions site</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>Yes — Safety</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>87%</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>AACSB-accredited College of Business. 10 undergraduate majors. No separate admission. Rolling admissions.</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>No separate admission process (General: https://www.appily.com/colleges/university-of-wisconsin-oshkosh)</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>North Dakota State University-Main Campus</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>373 (national)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>$9,868</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>$15,415</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>University general only</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>University admit only</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Mid-50% columns = university-wide (not College of Business). No EA/ED.</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>1010–1280</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
         <is>
           <t>In mid-50%</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>28–34</t>
-        </is>
-      </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>Below (-2 vs low)</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>Nov 1</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>Jan 15</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr">
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>19–25</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Above (+1 vs high)</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Aug 1</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
+      <c r="W36" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>Yes — Target</t>
-        </is>
-      </c>
-      <c r="W33" t="inlineStr">
-        <is>
-          <t>43%</t>
-        </is>
-      </c>
-      <c r="Y33" t="inlineStr">
-        <is>
-          <t>Daniels School of Business (formerly Krannert). Direct admission — indicate business on main app. Higher tuition differential: in-state ,428/yr, OOS ,230/yr. EA Nov 1 is priority for merit scholarships.</t>
-        </is>
-      </c>
-      <c r="Z33" t="inlineStr">
-        <is>
-          <t>No separate rate. Business tuition differential: in-state ,428, OOS ,230. (General: https://admissions.purdue.edu/become-student/class-profile/)</t>
-        </is>
-      </c>
-      <c r="AA33" t="inlineStr"/>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>Yes — Safety</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>College of Business — Barry Hall, downtown Fargo. 8 undergraduate majors. No separate admission requirements. ND reciprocity tuition for MN residents.</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>No separate admission process (General: https://www.appily.com/colleges/north-dakota-state-university-main-campus)</t>
+        </is>
+      </c>
+      <c r="AC36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Ashland University</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>R-MW #42 (regional)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>$31,210</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>University general only</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>University admit only</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>No published program mid-50%; general university admission. No EA/ED.</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>See admissions site</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>No — excluded</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>76.4%</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>Not yet researched</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>Tuition $31,210 exceeds budget $30,000</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>Auto stub — run scoped research for program-level rate (General: https://www.ashland.edu/ | Business: https://www.ashland.edu/)</t>
+        </is>
+      </c>
+      <c r="AC37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Heidelberg University</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>R-MW #71 (regional)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>$33,650</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>University general only</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>University admit only</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>No published program mid-50%; general university admission. No EA/ED.</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>See admissions site</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>No — excluded</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>85.8%</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>Not yet researched</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>Tuition $33,650 exceeds budget $30,000</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>Auto stub — run scoped research for program-level rate (General: https://www.heidelberg.edu/ | Business: https://www.heidelberg.edu/)</t>
+        </is>
+      </c>
+      <c r="AC38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>The University of Findlay</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>373 (national)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>$41,164</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>University general only</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>University admit only</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>No published program mid-50%; general university admission. No EA/ED.</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>See admissions site</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>No — excluded</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>83.4%</t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>Not yet researched</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>Tuition $41,164 exceeds budget $30,000</t>
+        </is>
+      </c>
+      <c r="AB39" t="inlineStr">
+        <is>
+          <t>Auto stub — run scoped research for program-level rate (General: https://www.findlay.edu/ | Business: https://www.findlay.edu/)</t>
+        </is>
+      </c>
+      <c r="AC39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
More fixes to use latest anthropic model and update related docs
</commit_message>
<xml_diff>
--- a/students/alex-sample/output/Alex - US College Selection.xlsx
+++ b/students/alex-sample/output/Alex - US College Selection.xlsx
@@ -2380,7 +2380,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>University of Wisconsin-Parkside</t>
+          <t>Youngstown State University</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2390,17 +2390,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>R-MW #118 (regional)</t>
+          <t>R-MW #99 (regional)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>$17,429</t>
+          <t>$11,113</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>$11,772</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>75.4%</t>
+          <t>84.5%</t>
         </is>
       </c>
       <c r="Z27" t="inlineStr">
@@ -2502,12 +2502,12 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>Out-of-state tuition $17,429/year.</t>
+          <t>In-state tuition $11,113/year — Ohio resident.</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>Auto stub — run scoped research for program-level rate (General: https://www.uwp.edu/ | Business: https://www.uwp.edu/)</t>
+          <t>Auto stub — run scoped research for program-level rate (General: https://ysu.edu/ | Business: https://ysu.edu/)</t>
         </is>
       </c>
       <c r="AC27" t="inlineStr"/>
@@ -2515,7 +2515,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>University of Wisconsin-Superior</t>
+          <t>University of Wisconsin-Parkside</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2525,17 +2525,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>R-MW #135 (regional)</t>
+          <t>R-MW #118 (regional)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>$16,726</t>
+          <t>$17,429</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>$12,220</t>
+          <t>$11,772</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>93.0%</t>
+          <t>75.4%</t>
         </is>
       </c>
       <c r="Z28" t="inlineStr">
@@ -2637,12 +2637,12 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>Out-of-state tuition $16,726/year.</t>
+          <t>Out-of-state tuition $17,429/year.</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>Auto stub — run scoped research for program-level rate (General: https://www.uwsuper.edu/ | Business: https://www.uwsuper.edu/)</t>
+          <t>Auto stub — run scoped research for program-level rate (General: https://www.uwp.edu/ | Business: https://www.uwp.edu/)</t>
         </is>
       </c>
       <c r="AC28" t="inlineStr"/>
@@ -2650,27 +2650,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Miami University-Oxford</t>
+          <t>University of Wisconsin-Superior</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>143 (national)</t>
+          <t>R-MW #135 (regional)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>$18,161</t>
+          <t>$16,726</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$12,220</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2762,7 +2762,7 @@
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>75.4%</t>
+          <t>93.0%</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
@@ -2772,12 +2772,12 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>In-state tuition $18,161/year — Ohio resident.</t>
+          <t>Out-of-state tuition $16,726/year.</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>Auto stub — run scoped research for program-level rate (General: https://miamioh.edu/ | Business: https://miamioh.edu/)</t>
+          <t>Auto stub — run scoped research for program-level rate (General: https://www.uwsuper.edu/ | Business: https://www.uwsuper.edu/)</t>
         </is>
       </c>
       <c r="AC29" t="inlineStr"/>
@@ -2785,22 +2785,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Kent State University at Kent</t>
+          <t>Miami University-Oxford</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>232 (national)</t>
+          <t>143 (national)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>$13,232</t>
+          <t>$18,161</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2897,7 +2897,7 @@
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>86.3%</t>
+          <t>75.4%</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
@@ -2907,12 +2907,12 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>In-state tuition $13,232/year — Ohio resident.</t>
+          <t>In-state tuition $18,161/year — Ohio resident.</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>Auto stub — run scoped research for program-level rate (General: https://www.kent.edu/ | Business: https://www.kent.edu/)</t>
+          <t>Auto stub — run scoped research for program-level rate (General: https://miamioh.edu/ | Business: https://miamioh.edu/)</t>
         </is>
       </c>
       <c r="AC30" t="inlineStr"/>
@@ -2920,7 +2920,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>University of Toledo</t>
+          <t>Kent State University at Kent</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2930,12 +2930,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>293 (national)</t>
+          <t>232 (national)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>$12,744</t>
+          <t>$13,232</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>92.0%</t>
+          <t>86.3%</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
@@ -3042,12 +3042,12 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>In-state tuition $12,744/year — Ohio resident.</t>
+          <t>In-state tuition $13,232/year — Ohio resident.</t>
         </is>
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>Auto stub — run scoped research for program-level rate (General: https://www.utoledo.edu/ | Business: https://www.utoledo.edu/)</t>
+          <t>Auto stub — run scoped research for program-level rate (General: https://www.kent.edu/ | Business: https://www.kent.edu/)</t>
         </is>
       </c>
       <c r="AC31" t="inlineStr"/>
@@ -3055,7 +3055,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>University of Wisconsin-Milwaukee</t>
+          <t>University of Toledo</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3065,17 +3065,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>301 (national)</t>
+          <t>293 (national)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>$23,516</t>
+          <t>$12,744</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>$15,014</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3167,17 +3167,22 @@
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>92.0%</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>Not yet researched</t>
         </is>
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>Sheldon B. Lubar College of Business. No separate admission. Rolling admissions. MN-WI reciprocity tuition for MN residents.</t>
+          <t>In-state tuition $12,744/year — Ohio resident.</t>
         </is>
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>No separate admission process (General: https://www.collegedata.com/college/University-of-Wisconsin-Milwaukee)</t>
+          <t>Auto stub — run scoped research for program-level rate (General: https://www.utoledo.edu/ | Business: https://www.utoledo.edu/)</t>
         </is>
       </c>
       <c r="AC32" t="inlineStr"/>
@@ -3185,7 +3190,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>University of Wisconsin-Oshkosh</t>
+          <t>University of Wisconsin-Milwaukee</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3195,17 +3200,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>352 (national)</t>
+          <t>301 (national)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>$16,444</t>
+          <t>$23,516</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>$14,305</t>
+          <t>$15,014</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3215,7 +3220,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3240,7 +3245,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Mid-50% columns = university-wide (not College of Business). No EA/ED.</t>
+          <t>No published program mid-50%; general university admission. No EA/ED.</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -3265,12 +3270,12 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>19–24</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Above (+2 vs high)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
@@ -3297,17 +3302,17 @@
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>AACSB-accredited College of Business. 10 undergraduate majors. No separate admission. Rolling admissions.</t>
+          <t>Sheldon B. Lubar College of Business. No separate admission. Rolling admissions. MN-WI reciprocity tuition for MN residents.</t>
         </is>
       </c>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>No separate admission process (General: https://www.appily.com/colleges/university-of-wisconsin-oshkosh)</t>
+          <t>No separate admission process (General: https://www.collegedata.com/college/University-of-Wisconsin-Milwaukee)</t>
         </is>
       </c>
       <c r="AC33" t="inlineStr"/>
@@ -3315,7 +3320,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>North Dakota State University-Main Campus</t>
+          <t>University of Wisconsin-Oshkosh</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3325,17 +3330,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>373 (national)</t>
+          <t>352 (national)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>$9,868</t>
+          <t>$16,444</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>$15,415</t>
+          <t>$14,305</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3345,7 +3350,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -3385,29 +3390,29 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>1010–1280</t>
+          <t>—</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>In mid-50%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>19–25</t>
+          <t>19–24</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Above (+1 vs high)</t>
+          <t>Above (+2 vs high)</t>
         </is>
       </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr"/>
       <c r="U34" t="inlineStr">
         <is>
-          <t>Aug 1</t>
+          <t>See admissions site</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
@@ -3427,17 +3432,17 @@
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>87%</t>
         </is>
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>College of Business — Barry Hall, downtown Fargo. 8 undergraduate majors. No separate admission requirements. ND reciprocity tuition for MN residents.</t>
+          <t>AACSB-accredited College of Business. 10 undergraduate majors. No separate admission. Rolling admissions.</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>No separate admission process (General: https://www.appily.com/colleges/north-dakota-state-university-main-campus)</t>
+          <t>No separate admission process (General: https://www.appily.com/colleges/university-of-wisconsin-oshkosh)</t>
         </is>
       </c>
       <c r="AC34" t="inlineStr"/>
@@ -3445,37 +3450,37 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Western Reserve Academy</t>
+          <t>North Dakota State University-Main Campus</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>51 (national)</t>
+          <t>373 (national)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>$0</t>
+          <t>$9,868</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$15,415</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3500,7 +3505,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>No published program mid-50%; general university admission. No EA/ED.</t>
+          <t>Mid-50% columns = university-wide (not College of Business). No EA/ED.</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -3515,29 +3520,29 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1010–1280</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>In mid-50%</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>19–25</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Above (+1 vs high)</t>
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr">
         <is>
-          <t>See admissions site</t>
+          <t>Aug 1</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
@@ -3552,27 +3557,22 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>Yes — Target</t>
+          <t>Yes — Safety</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>Not yet researched</t>
-        </is>
-      </c>
-      <c r="Z35" t="inlineStr">
-        <is>
-          <t>Not yet researched</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>In-state tuition $0/year — Ohio resident.</t>
+          <t>College of Business — Barry Hall, downtown Fargo. 8 undergraduate majors. No separate admission requirements. ND reciprocity tuition for MN residents.</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>Auto stub — run scoped research for program-level rate (General: https://collegescorecard.ed.gov/ | Business: https://collegescorecard.ed.gov/)</t>
+          <t>No separate admission process (General: https://www.appily.com/colleges/north-dakota-state-university-main-campus)</t>
         </is>
       </c>
       <c r="AC35" t="inlineStr"/>
@@ -3580,7 +3580,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>John Carroll University</t>
+          <t>Western Reserve Academy</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3590,12 +3590,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>R-MW #2 (regional)</t>
+          <t>51 (national)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>$50,500</t>
+          <t>$0</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3682,17 +3682,17 @@
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>No — excluded</t>
+          <t>Yes — Target</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>80.9%</t>
+          <t>Not yet researched</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr">
@@ -3702,12 +3702,12 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>Tuition $50,500 exceeds budget $25,000</t>
+          <t>In-state tuition $0/year — Ohio resident.</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>Auto stub — run scoped research for program-level rate (General: https://jcu.edu/ | Business: https://jcu.edu/)</t>
+          <t>Auto stub — run scoped research for program-level rate (General: https://collegescorecard.ed.gov/ | Business: https://collegescorecard.ed.gov/)</t>
         </is>
       </c>
       <c r="AC36" t="inlineStr"/>
@@ -3715,22 +3715,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ashland University</t>
+          <t>Shawnee State University</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>R-MW #42 (regional)</t>
+          <t>R-MW #112 (regional)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>$31,210</t>
+          <t>$10,626</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3817,17 +3817,17 @@
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>No — excluded</t>
+          <t>Yes — Target</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>76.4%</t>
+          <t>Not yet researched</t>
         </is>
       </c>
       <c r="Z37" t="inlineStr">
@@ -3837,12 +3837,12 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>Tuition $31,210 exceeds budget $25,000</t>
+          <t>In-state tuition $10,626/year — Ohio resident.</t>
         </is>
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>Auto stub — run scoped research for program-level rate (General: https://www.ashland.edu/ | Business: https://www.ashland.edu/)</t>
+          <t>Auto stub — run scoped research for program-level rate (General: https://www.shawnee.edu/ | Business: https://www.shawnee.edu/)</t>
         </is>
       </c>
       <c r="AC37" t="inlineStr"/>
@@ -3850,7 +3850,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Case Western Reserve University</t>
+          <t>Ashland University</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3860,12 +3860,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>51 (national)</t>
+          <t>R-MW #42 (regional)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>$66,608</t>
+          <t>$31,210</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>36.5%</t>
+          <t>76.4%</t>
         </is>
       </c>
       <c r="Z38" t="inlineStr">
@@ -3972,12 +3972,12 @@
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>Tuition $66,608 exceeds budget $25,000</t>
+          <t>Tuition $31,210 exceeds budget $25,000</t>
         </is>
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>Auto stub — run scoped research for program-level rate (General: https://www.case.edu/ | Business: https://www.case.edu/)</t>
+          <t>Auto stub — run scoped research for program-level rate (General: https://www.ashland.edu/ | Business: https://www.ashland.edu/)</t>
         </is>
       </c>
       <c r="AC38" t="inlineStr"/>
@@ -3985,7 +3985,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Tiffin University</t>
+          <t>Case Western Reserve University</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3995,22 +3995,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>R-MW #138 (regional)</t>
+          <t>51 (national)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>$34,790</t>
+          <t>$66,608</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>$26,500</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4097,7 +4097,7 @@
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>36.5%</t>
         </is>
       </c>
       <c r="Z39" t="inlineStr">
@@ -4107,12 +4107,12 @@
       </c>
       <c r="AA39" t="inlineStr">
         <is>
-          <t>Sticker $34,790 and avg net price $26,500 both exceed budget $25,000</t>
+          <t>Tuition $66,608 exceeds budget $25,000</t>
         </is>
       </c>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>Auto stub — run scoped research for program-level rate (General: https://www.tiffin.edu/ | Business: https://www.tiffin.edu/)</t>
+          <t>Auto stub — run scoped research for program-level rate (General: https://www.case.edu/ | Business: https://www.case.edu/)</t>
         </is>
       </c>
       <c r="AC39" t="inlineStr"/>

</xml_diff>